<commit_message>
v2.4 imu calibrated、R1 radio map
</commit_message>
<xml_diff>
--- a/py/figure/test1/test1_error.xlsx
+++ b/py/figure/test1/test1_error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2023_IPIN_Competition_Track03\py\figure\test1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CCC30A5-9573-47E5-B431-D667BEC41C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71270108-596A-48C5-83AE-CAB94A72F216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{27DAA2EC-07AC-43C6-81D7-23A2318EAE70}"/>
+    <workbookView xWindow="15972" yWindow="1800" windowWidth="23040" windowHeight="12204" xr2:uid="{27DAA2EC-07AC-43C6-81D7-23A2318EAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -513,6 +513,9 @@
       <c r="B6" s="1">
         <v>6.34</v>
       </c>
+      <c r="D6" s="1">
+        <v>4.5999999999999996</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -521,6 +524,9 @@
       <c r="B7" s="1">
         <v>4.92</v>
       </c>
+      <c r="D7" s="1">
+        <v>3.67</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -529,6 +535,9 @@
       <c r="B8" s="1">
         <v>4</v>
       </c>
+      <c r="D8" s="1">
+        <v>2.78</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -536,6 +545,9 @@
       </c>
       <c r="B9" s="1">
         <v>27.5</v>
+      </c>
+      <c r="D9" s="1">
+        <v>11.8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>